<commit_message>
Update attendance sheets for EDA and Introduction to Programming for the 2026-27 academic year
</commit_message>
<xml_diff>
--- a/Folha_de_Presencas_EDA_2026-27_28jan2026.xlsx
+++ b/Folha_de_Presencas_EDA_2026-27_28jan2026.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
   <si>
     <t>REGISTO DE PRESENÇAS</t>
   </si>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>x</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
   <si>
     <t>13439</t>
@@ -2015,7 +2018,9 @@
         <v>17</v>
       </c>
       <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
+      <c r="E8" s="18" t="s">
+        <v>18</v>
+      </c>
       <c r="F8" s="18"/>
       <c r="G8" s="18"/>
       <c r="H8" s="18"/>
@@ -2029,7 +2034,7 @@
       <c r="P8" s="19"/>
       <c r="Q8" s="20">
         <f>COUNTIF(C8:P8,"X")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R8" s="21">
         <f t="shared" ref="R8:R13" si="0">COUNTIF(C8:P8,"F")</f>
@@ -2042,16 +2047,18 @@
     </row>
     <row r="9" ht="34" customHeight="1" spans="1:19">
       <c r="A9" s="23" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C9" s="25" t="s">
         <v>17</v>
       </c>
       <c r="D9" s="26"/>
-      <c r="E9" s="26"/>
+      <c r="E9" s="26" t="s">
+        <v>18</v>
+      </c>
       <c r="F9" s="26"/>
       <c r="G9" s="26"/>
       <c r="H9" s="26"/>
@@ -2065,7 +2072,7 @@
       <c r="P9" s="27"/>
       <c r="Q9" s="28">
         <f t="shared" ref="Q9:Q13" si="2">COUNTIF(C9:P9,"X")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R9" s="29">
         <f t="shared" si="0"/>
@@ -2078,10 +2085,10 @@
     </row>
     <row r="10" ht="34" customHeight="1" spans="1:19">
       <c r="A10" s="31" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B10" s="32" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C10" s="25" t="s">
         <v>17</v>
@@ -2116,10 +2123,10 @@
     </row>
     <row r="11" ht="34" customHeight="1" spans="1:19">
       <c r="A11" s="23" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C11" s="25" t="s">
         <v>17</v>
@@ -2156,10 +2163,10 @@
     </row>
     <row r="12" ht="34" customHeight="1" spans="1:19">
       <c r="A12" s="33" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" s="34" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C12" s="35" t="s">
         <v>17</v>
@@ -2192,10 +2199,10 @@
     </row>
     <row r="13" ht="26" customHeight="1" spans="1:19">
       <c r="A13" s="23" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C13" s="25" t="s">
         <v>17</v>
@@ -2252,7 +2259,7 @@
     <row r="15" ht="25" customHeight="1" spans="1:19">
       <c r="A15" s="1"/>
       <c r="B15" s="40" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C15" s="41">
         <f>COUNTIF(C8:C12,"X")+COUNTIF(C8:C12,"F")+COUNTIF(C8:C12,"J")</f>
@@ -2264,7 +2271,7 @@
       </c>
       <c r="E15" s="41">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F15" s="41">
         <f t="shared" si="3"/>
@@ -2312,7 +2319,7 @@
       </c>
       <c r="Q15" s="41">
         <f>SUM(Q8:Q12)</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R15" s="41">
         <f>SUM(R8:R12)</f>
@@ -2346,7 +2353,7 @@
     </row>
     <row r="17" ht="20" customHeight="1" spans="1:19">
       <c r="A17" s="42" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
@@ -2369,7 +2376,7 @@
     </row>
     <row r="18" ht="20" customHeight="1" spans="1:19">
       <c r="A18" s="43" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -2392,7 +2399,7 @@
     </row>
     <row r="19" ht="20" customHeight="1" spans="1:19">
       <c r="A19" s="44" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>

</xml_diff>

<commit_message>
Update attendance sheet for EDA 2026-27
</commit_message>
<xml_diff>
--- a/Folha_de_Presencas_EDA_2026-27_28jan2026.xlsx
+++ b/Folha_de_Presencas_EDA_2026-27_28jan2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6800"/>
+    <workbookView windowWidth="19200" windowHeight="6200"/>
   </bookViews>
   <sheets>
     <sheet name="Presenças" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
   <si>
     <t>REGISTO DE PRESENÇAS</t>
   </si>
@@ -2059,7 +2059,9 @@
       <c r="E9" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="26"/>
+      <c r="F9" s="26" t="s">
+        <v>18</v>
+      </c>
       <c r="G9" s="26"/>
       <c r="H9" s="26"/>
       <c r="I9" s="26"/>
@@ -2072,7 +2074,7 @@
       <c r="P9" s="27"/>
       <c r="Q9" s="28">
         <f t="shared" ref="Q9:Q13" si="2">COUNTIF(C9:P9,"X")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R9" s="29">
         <f t="shared" si="0"/>
@@ -2137,7 +2139,9 @@
       <c r="E11" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="F11" s="26"/>
+      <c r="F11" s="26" t="s">
+        <v>18</v>
+      </c>
       <c r="G11" s="26"/>
       <c r="H11" s="26"/>
       <c r="I11" s="26"/>
@@ -2150,7 +2154,7 @@
       <c r="P11" s="27"/>
       <c r="Q11" s="28">
         <f t="shared" si="2"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R11" s="29">
         <f t="shared" si="0"/>
@@ -2211,7 +2215,9 @@
         <v>17</v>
       </c>
       <c r="E13" s="26"/>
-      <c r="F13" s="26"/>
+      <c r="F13" s="26" t="s">
+        <v>18</v>
+      </c>
       <c r="G13" s="26"/>
       <c r="H13" s="26"/>
       <c r="I13" s="26"/>
@@ -2224,7 +2230,7 @@
       <c r="P13" s="27"/>
       <c r="Q13" s="28">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R13" s="29">
         <f t="shared" si="0"/>
@@ -2275,7 +2281,7 @@
       </c>
       <c r="F15" s="41">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G15" s="41">
         <f t="shared" si="3"/>
@@ -2319,7 +2325,7 @@
       </c>
       <c r="Q15" s="41">
         <f>SUM(Q8:Q12)</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="R15" s="41">
         <f>SUM(R8:R12)</f>

</xml_diff>